<commit_message>
Correcting water evaporation unit error for sizing (kg instead of m3)
</commit_message>
<xml_diff>
--- a/datasets/weaving/inventory-brightway.xlsx
+++ b/datasets/weaving/inventory-brightway.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vincentcarrieres/carbonfact/lca/lca/notebooks/science/Carbonfact database/Weaving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE19F7C-6B81-614C-8BE5-0217CF69FCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0F4C8E-3E25-224B-B573-9AF39E17026C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4540" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16940" yWindow="-21000" windowWidth="16300" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1129,7 +1129,7 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>1.008554631</v>
+        <v>1.0085546309999999E-3</v>
       </c>
       <c r="D34" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Correcting water evaporation unit error for sizing (kg instead of m3) (#31)
Water evaporation to air was initially declared in kg in the LCI of
`Fabric Sizing, Natural Fibres` process, and mapped in m3 in
`brightway-inventory` (native unit of the biosphere flow in ecoinvent),
significantly overestimating impact on WTU indicator.

A fix was applied, reducing WTU impacts of affected processes between
-95% and -99%. See diff analysis attached

[Weaving_Diff_Analysis_200426.xlsx](https://github.com/user-attachments/files/27250040/Weaving_Diff_Analysis_200426.xlsx)
</commit_message>
<xml_diff>
--- a/datasets/weaving/inventory-brightway.xlsx
+++ b/datasets/weaving/inventory-brightway.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vincentcarrieres/carbonfact/lca/lca/notebooks/science/Carbonfact database/Weaving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE19F7C-6B81-614C-8BE5-0217CF69FCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0F4C8E-3E25-224B-B573-9AF39E17026C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4540" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16940" yWindow="-21000" windowWidth="16300" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1129,7 +1129,7 @@
         <v>48</v>
       </c>
       <c r="B34">
-        <v>1.008554631</v>
+        <v>1.0085546309999999E-3</v>
       </c>
       <c r="D34" t="s">
         <v>7</v>

</xml_diff>